<commit_message>
feat: ignore 'Specify' line weights when determining 'Plots Same As' and update JVC1.xlsx.
</commit_message>
<xml_diff>
--- a/JVC1_optimized.xlsx
+++ b/JVC1_optimized.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\swalker\dev\ctb-translator\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4129CBCD-93FE-4212-95C7-96F39979120F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CTB Data" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1771" uniqueCount="714">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1509" uniqueCount="714">
   <si>
     <t>Color</t>
   </si>
@@ -2161,8 +2167,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="221">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="221" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5291,13 +5297,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -5335,7 +5349,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -5369,6 +5383,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -5403,9 +5418,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -5578,19 +5594,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G256"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" customWidth="1"/>
-    <col min="2" max="3" width="15.7109375" customWidth="1"/>
-    <col min="4" max="4" width="10.7109375" customWidth="1"/>
-    <col min="5" max="5" width="8.7109375" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" customWidth="1"/>
-    <col min="7" max="7" width="50.7109375" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="255.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5613,7 +5630,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -5636,7 +5653,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -5659,7 +5676,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -5682,7 +5699,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -5705,7 +5722,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -5728,7 +5745,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -5751,7 +5768,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -5774,7 +5791,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -5797,7 +5814,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -5820,7 +5837,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -5843,7 +5860,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -5866,7 +5883,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>18</v>
       </c>
@@ -5889,7 +5906,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>19</v>
       </c>
@@ -5912,7 +5929,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -5935,7 +5952,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>21</v>
       </c>
@@ -5958,7 +5975,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>22</v>
       </c>
@@ -5981,7 +5998,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -6001,7 +6018,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -6024,7 +6041,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>25</v>
       </c>
@@ -6044,7 +6061,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>26</v>
       </c>
@@ -6064,7 +6081,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>27</v>
       </c>
@@ -6087,7 +6104,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>28</v>
       </c>
@@ -6110,7 +6127,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="24" spans="1:7">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>29</v>
       </c>
@@ -6133,7 +6150,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="25" spans="1:7">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>30</v>
       </c>
@@ -6156,7 +6173,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>31</v>
       </c>
@@ -6179,7 +6196,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>32</v>
       </c>
@@ -6202,7 +6219,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="28" spans="1:7">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>33</v>
       </c>
@@ -6225,7 +6242,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="29" spans="1:7">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>34</v>
       </c>
@@ -6248,7 +6265,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="30" spans="1:7">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>35</v>
       </c>
@@ -6271,7 +6288,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="31" spans="1:7">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>36</v>
       </c>
@@ -6294,7 +6311,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="32" spans="1:7">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>37</v>
       </c>
@@ -6317,7 +6334,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="33" spans="1:7">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>38</v>
       </c>
@@ -6340,7 +6357,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="34" spans="1:7">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>39</v>
       </c>
@@ -6363,7 +6380,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="35" spans="1:7">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>40</v>
       </c>
@@ -6386,7 +6403,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="36" spans="1:7">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>41</v>
       </c>
@@ -6409,7 +6426,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="37" spans="1:7">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>42</v>
       </c>
@@ -6432,7 +6449,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="38" spans="1:7">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>43</v>
       </c>
@@ -6455,7 +6472,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="39" spans="1:7">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>44</v>
       </c>
@@ -6478,7 +6495,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="40" spans="1:7">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>45</v>
       </c>
@@ -6501,7 +6518,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="41" spans="1:7">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>46</v>
       </c>
@@ -6524,7 +6541,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="42" spans="1:7">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>47</v>
       </c>
@@ -6547,7 +6564,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="43" spans="1:7">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>48</v>
       </c>
@@ -6570,7 +6587,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="44" spans="1:7">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>49</v>
       </c>
@@ -6593,7 +6610,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="45" spans="1:7">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>50</v>
       </c>
@@ -6616,7 +6633,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="46" spans="1:7">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>51</v>
       </c>
@@ -6639,7 +6656,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="47" spans="1:7">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>52</v>
       </c>
@@ -6662,7 +6679,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="48" spans="1:7">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>53</v>
       </c>
@@ -6685,7 +6702,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="49" spans="1:7">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>54</v>
       </c>
@@ -6708,7 +6725,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="50" spans="1:7">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>55</v>
       </c>
@@ -6731,7 +6748,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="51" spans="1:7">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>56</v>
       </c>
@@ -6754,7 +6771,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="52" spans="1:7">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>57</v>
       </c>
@@ -6777,7 +6794,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="53" spans="1:7">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>58</v>
       </c>
@@ -6800,7 +6817,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="54" spans="1:7">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>59</v>
       </c>
@@ -6823,7 +6840,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="55" spans="1:7">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>60</v>
       </c>
@@ -6846,7 +6863,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="56" spans="1:7">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>61</v>
       </c>
@@ -6869,7 +6886,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="57" spans="1:7">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>62</v>
       </c>
@@ -6892,7 +6909,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="58" spans="1:7">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>63</v>
       </c>
@@ -6915,7 +6932,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="59" spans="1:7">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>64</v>
       </c>
@@ -6938,7 +6955,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="60" spans="1:7">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>65</v>
       </c>
@@ -6961,7 +6978,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="61" spans="1:7">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>66</v>
       </c>
@@ -6984,7 +7001,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="62" spans="1:7">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>67</v>
       </c>
@@ -7007,7 +7024,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="63" spans="1:7">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>68</v>
       </c>
@@ -7030,7 +7047,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="64" spans="1:7">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>69</v>
       </c>
@@ -7053,7 +7070,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="65" spans="1:7">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>70</v>
       </c>
@@ -7076,7 +7093,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="66" spans="1:7">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>71</v>
       </c>
@@ -7099,7 +7116,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="67" spans="1:7">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>72</v>
       </c>
@@ -7122,7 +7139,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="68" spans="1:7">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>73</v>
       </c>
@@ -7145,7 +7162,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="69" spans="1:7">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>74</v>
       </c>
@@ -7165,7 +7182,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="70" spans="1:7">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>75</v>
       </c>
@@ -7188,7 +7205,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="71" spans="1:7">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>76</v>
       </c>
@@ -7211,7 +7228,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="72" spans="1:7">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>77</v>
       </c>
@@ -7234,7 +7251,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="73" spans="1:7">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>78</v>
       </c>
@@ -7257,7 +7274,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="74" spans="1:7">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>79</v>
       </c>
@@ -7280,7 +7297,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="75" spans="1:7">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>80</v>
       </c>
@@ -7303,7 +7320,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="76" spans="1:7">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>81</v>
       </c>
@@ -7323,7 +7340,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="77" spans="1:7">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>82</v>
       </c>
@@ -7346,7 +7363,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="78" spans="1:7">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>83</v>
       </c>
@@ -7369,7 +7386,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="79" spans="1:7">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>84</v>
       </c>
@@ -7392,7 +7409,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="80" spans="1:7">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>85</v>
       </c>
@@ -7415,7 +7432,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="81" spans="1:7">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>86</v>
       </c>
@@ -7438,7 +7455,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="82" spans="1:7">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>87</v>
       </c>
@@ -7461,7 +7478,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="83" spans="1:7">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>88</v>
       </c>
@@ -7484,7 +7501,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="84" spans="1:7">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>89</v>
       </c>
@@ -7507,7 +7524,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="85" spans="1:7">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>90</v>
       </c>
@@ -7530,7 +7547,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="86" spans="1:7">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>91</v>
       </c>
@@ -7553,7 +7570,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="87" spans="1:7">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>92</v>
       </c>
@@ -7576,7 +7593,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="88" spans="1:7">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>93</v>
       </c>
@@ -7599,7 +7616,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="89" spans="1:7">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>94</v>
       </c>
@@ -7622,7 +7639,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="90" spans="1:7">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>95</v>
       </c>
@@ -7645,7 +7662,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="91" spans="1:7">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>96</v>
       </c>
@@ -7668,7 +7685,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="92" spans="1:7">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>97</v>
       </c>
@@ -7691,7 +7708,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="93" spans="1:7">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>98</v>
       </c>
@@ -7714,7 +7731,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="94" spans="1:7">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>99</v>
       </c>
@@ -7737,7 +7754,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="95" spans="1:7">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>100</v>
       </c>
@@ -7760,7 +7777,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="96" spans="1:7">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>101</v>
       </c>
@@ -7783,7 +7800,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="97" spans="1:7">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>102</v>
       </c>
@@ -7806,7 +7823,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="98" spans="1:7">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>103</v>
       </c>
@@ -7829,7 +7846,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="99" spans="1:7">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>104</v>
       </c>
@@ -7852,7 +7869,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="100" spans="1:7">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>105</v>
       </c>
@@ -7875,7 +7892,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="101" spans="1:7">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>106</v>
       </c>
@@ -7895,7 +7912,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="102" spans="1:7">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>107</v>
       </c>
@@ -7918,7 +7935,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="103" spans="1:7">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>108</v>
       </c>
@@ -7941,7 +7958,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="104" spans="1:7">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>109</v>
       </c>
@@ -7964,7 +7981,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="105" spans="1:7">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>110</v>
       </c>
@@ -7987,7 +8004,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="106" spans="1:7">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>111</v>
       </c>
@@ -8010,7 +8027,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="107" spans="1:7">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>112</v>
       </c>
@@ -8033,7 +8050,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="108" spans="1:7">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>113</v>
       </c>
@@ -8056,7 +8073,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="109" spans="1:7">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>114</v>
       </c>
@@ -8079,7 +8096,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="110" spans="1:7">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>115</v>
       </c>
@@ -8102,7 +8119,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="111" spans="1:7">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>116</v>
       </c>
@@ -8125,7 +8142,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="112" spans="1:7">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>117</v>
       </c>
@@ -8148,7 +8165,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="113" spans="1:7">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>118</v>
       </c>
@@ -8171,7 +8188,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="114" spans="1:7">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>119</v>
       </c>
@@ -8194,7 +8211,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="115" spans="1:7">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>120</v>
       </c>
@@ -8217,7 +8234,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="116" spans="1:7">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>121</v>
       </c>
@@ -8240,7 +8257,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="117" spans="1:7">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>122</v>
       </c>
@@ -8263,7 +8280,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="118" spans="1:7">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>123</v>
       </c>
@@ -8286,7 +8303,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="119" spans="1:7">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>124</v>
       </c>
@@ -8309,7 +8326,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="120" spans="1:7">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>125</v>
       </c>
@@ -8332,7 +8349,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="121" spans="1:7">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>126</v>
       </c>
@@ -8355,7 +8372,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="122" spans="1:7">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>127</v>
       </c>
@@ -8378,7 +8395,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="123" spans="1:7">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>128</v>
       </c>
@@ -8401,7 +8418,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="124" spans="1:7">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>129</v>
       </c>
@@ -8424,7 +8441,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="125" spans="1:7">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>130</v>
       </c>
@@ -8447,7 +8464,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="126" spans="1:7">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>131</v>
       </c>
@@ -8470,7 +8487,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="127" spans="1:7">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>132</v>
       </c>
@@ -8493,7 +8510,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="128" spans="1:7">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>133</v>
       </c>
@@ -8516,7 +8533,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="129" spans="1:7">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>134</v>
       </c>
@@ -8539,7 +8556,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="130" spans="1:7">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>135</v>
       </c>
@@ -8562,7 +8579,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="131" spans="1:7">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>136</v>
       </c>
@@ -8585,7 +8602,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="132" spans="1:7">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>137</v>
       </c>
@@ -8608,7 +8625,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="133" spans="1:7">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>138</v>
       </c>
@@ -8631,7 +8648,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="134" spans="1:7">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>139</v>
       </c>
@@ -8654,7 +8671,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="135" spans="1:7">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>140</v>
       </c>
@@ -8677,7 +8694,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="136" spans="1:7">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>141</v>
       </c>
@@ -8700,7 +8717,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="137" spans="1:7">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>142</v>
       </c>
@@ -8723,7 +8740,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="138" spans="1:7">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>143</v>
       </c>
@@ -8746,7 +8763,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="139" spans="1:7">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>144</v>
       </c>
@@ -8769,7 +8786,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="140" spans="1:7">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>145</v>
       </c>
@@ -8792,7 +8809,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="141" spans="1:7">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>146</v>
       </c>
@@ -8812,7 +8829,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="142" spans="1:7">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>147</v>
       </c>
@@ -8835,7 +8852,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="143" spans="1:7">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>148</v>
       </c>
@@ -8858,7 +8875,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="144" spans="1:7">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>149</v>
       </c>
@@ -8881,7 +8898,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="145" spans="1:7">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>150</v>
       </c>
@@ -8904,7 +8921,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="146" spans="1:7">
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>151</v>
       </c>
@@ -8927,7 +8944,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="147" spans="1:7">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>152</v>
       </c>
@@ -8950,7 +8967,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="148" spans="1:7">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>153</v>
       </c>
@@ -8973,7 +8990,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="149" spans="1:7">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>154</v>
       </c>
@@ -8996,7 +9013,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="150" spans="1:7">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>155</v>
       </c>
@@ -9019,7 +9036,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="151" spans="1:7">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>156</v>
       </c>
@@ -9042,7 +9059,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="152" spans="1:7">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>157</v>
       </c>
@@ -9065,7 +9082,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="153" spans="1:7">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>158</v>
       </c>
@@ -9088,7 +9105,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="154" spans="1:7">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>159</v>
       </c>
@@ -9111,7 +9128,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="155" spans="1:7">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>160</v>
       </c>
@@ -9131,7 +9148,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="156" spans="1:7">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>161</v>
       </c>
@@ -9154,7 +9171,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="157" spans="1:7">
+    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>162</v>
       </c>
@@ -9177,7 +9194,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="158" spans="1:7">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>163</v>
       </c>
@@ -9200,7 +9217,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="159" spans="1:7">
+    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>164</v>
       </c>
@@ -9223,7 +9240,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="160" spans="1:7">
+    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>165</v>
       </c>
@@ -9246,7 +9263,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="161" spans="1:7">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>166</v>
       </c>
@@ -9266,7 +9283,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="162" spans="1:7">
+    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>167</v>
       </c>
@@ -9289,7 +9306,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="163" spans="1:7">
+    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>168</v>
       </c>
@@ -9312,7 +9329,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="164" spans="1:7">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>169</v>
       </c>
@@ -9335,7 +9352,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="165" spans="1:7">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>170</v>
       </c>
@@ -9358,7 +9375,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="166" spans="1:7">
+    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>171</v>
       </c>
@@ -9381,7 +9398,7 @@
         <v>647</v>
       </c>
     </row>
-    <row r="167" spans="1:7">
+    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>172</v>
       </c>
@@ -9404,7 +9421,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="168" spans="1:7">
+    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>173</v>
       </c>
@@ -9427,7 +9444,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="169" spans="1:7">
+    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>174</v>
       </c>
@@ -9450,7 +9467,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="170" spans="1:7">
+    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>175</v>
       </c>
@@ -9473,7 +9490,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="171" spans="1:7">
+    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>176</v>
       </c>
@@ -9496,7 +9513,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="172" spans="1:7">
+    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>177</v>
       </c>
@@ -9519,7 +9536,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="173" spans="1:7">
+    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>178</v>
       </c>
@@ -9542,7 +9559,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="174" spans="1:7">
+    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>179</v>
       </c>
@@ -9562,7 +9579,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="175" spans="1:7">
+    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>180</v>
       </c>
@@ -9585,7 +9602,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="176" spans="1:7">
+    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>181</v>
       </c>
@@ -9608,7 +9625,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="177" spans="1:7">
+    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>182</v>
       </c>
@@ -9631,7 +9648,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="178" spans="1:7">
+    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>183</v>
       </c>
@@ -9654,7 +9671,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="179" spans="1:7">
+    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>184</v>
       </c>
@@ -9674,7 +9691,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="180" spans="1:7">
+    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>185</v>
       </c>
@@ -9697,7 +9714,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="181" spans="1:7">
+    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>186</v>
       </c>
@@ -9720,7 +9737,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="182" spans="1:7">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>187</v>
       </c>
@@ -9743,7 +9760,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="183" spans="1:7">
+    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>188</v>
       </c>
@@ -9766,7 +9783,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="184" spans="1:7">
+    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>189</v>
       </c>
@@ -9789,7 +9806,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="185" spans="1:7">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>190</v>
       </c>
@@ -9812,7 +9829,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="186" spans="1:7">
+    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>191</v>
       </c>
@@ -9835,7 +9852,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="187" spans="1:7">
+    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>192</v>
       </c>
@@ -9858,7 +9875,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="188" spans="1:7">
+    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>193</v>
       </c>
@@ -9881,7 +9898,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="189" spans="1:7">
+    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>194</v>
       </c>
@@ -9904,7 +9921,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="190" spans="1:7">
+    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>195</v>
       </c>
@@ -9927,7 +9944,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="191" spans="1:7">
+    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>196</v>
       </c>
@@ -9950,7 +9967,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="192" spans="1:7">
+    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>197</v>
       </c>
@@ -9973,7 +9990,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="193" spans="1:7">
+    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>198</v>
       </c>
@@ -9996,7 +10013,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="194" spans="1:7">
+    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>199</v>
       </c>
@@ -10019,7 +10036,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="195" spans="1:7">
+    <row r="195" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>200</v>
       </c>
@@ -10042,7 +10059,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="196" spans="1:7">
+    <row r="196" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>201</v>
       </c>
@@ -10065,7 +10082,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="197" spans="1:7">
+    <row r="197" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>202</v>
       </c>
@@ -10088,7 +10105,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="198" spans="1:7">
+    <row r="198" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>203</v>
       </c>
@@ -10111,7 +10128,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="199" spans="1:7">
+    <row r="199" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>204</v>
       </c>
@@ -10134,7 +10151,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="200" spans="1:7">
+    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>205</v>
       </c>
@@ -10157,7 +10174,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="201" spans="1:7">
+    <row r="201" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>206</v>
       </c>
@@ -10180,7 +10197,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="202" spans="1:7">
+    <row r="202" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>207</v>
       </c>
@@ -10203,7 +10220,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="203" spans="1:7">
+    <row r="203" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>208</v>
       </c>
@@ -10226,7 +10243,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="204" spans="1:7">
+    <row r="204" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>209</v>
       </c>
@@ -10249,7 +10266,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="205" spans="1:7">
+    <row r="205" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>210</v>
       </c>
@@ -10272,7 +10289,7 @@
         <v>681</v>
       </c>
     </row>
-    <row r="206" spans="1:7">
+    <row r="206" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>211</v>
       </c>
@@ -10295,7 +10312,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="207" spans="1:7">
+    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>212</v>
       </c>
@@ -10318,7 +10335,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="208" spans="1:7">
+    <row r="208" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>213</v>
       </c>
@@ -10341,7 +10358,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="209" spans="1:7">
+    <row r="209" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>214</v>
       </c>
@@ -10361,7 +10378,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="210" spans="1:7">
+    <row r="210" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>215</v>
       </c>
@@ -10384,7 +10401,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="211" spans="1:7">
+    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>216</v>
       </c>
@@ -10407,7 +10424,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="212" spans="1:7">
+    <row r="212" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>217</v>
       </c>
@@ -10430,7 +10447,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="213" spans="1:7">
+    <row r="213" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>218</v>
       </c>
@@ -10453,7 +10470,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="214" spans="1:7">
+    <row r="214" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>219</v>
       </c>
@@ -10476,7 +10493,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="215" spans="1:7">
+    <row r="215" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>220</v>
       </c>
@@ -10499,7 +10516,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="216" spans="1:7">
+    <row r="216" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>221</v>
       </c>
@@ -10522,7 +10539,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="217" spans="1:7">
+    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>222</v>
       </c>
@@ -10545,7 +10562,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="218" spans="1:7">
+    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>223</v>
       </c>
@@ -10568,7 +10585,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="219" spans="1:7">
+    <row r="219" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
         <v>224</v>
       </c>
@@ -10591,7 +10608,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="220" spans="1:7">
+    <row r="220" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>225</v>
       </c>
@@ -10614,7 +10631,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="221" spans="1:7">
+    <row r="221" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>226</v>
       </c>
@@ -10637,7 +10654,7 @@
         <v>695</v>
       </c>
     </row>
-    <row r="222" spans="1:7">
+    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>227</v>
       </c>
@@ -10660,7 +10677,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="223" spans="1:7">
+    <row r="223" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>228</v>
       </c>
@@ -10683,7 +10700,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="224" spans="1:7">
+    <row r="224" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>229</v>
       </c>
@@ -10706,7 +10723,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="225" spans="1:7">
+    <row r="225" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>230</v>
       </c>
@@ -10729,7 +10746,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="226" spans="1:7">
+    <row r="226" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>231</v>
       </c>
@@ -10749,7 +10766,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="227" spans="1:7">
+    <row r="227" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>232</v>
       </c>
@@ -10772,7 +10789,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="228" spans="1:7">
+    <row r="228" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>233</v>
       </c>
@@ -10792,7 +10809,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="229" spans="1:7">
+    <row r="229" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>234</v>
       </c>
@@ -10815,7 +10832,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="230" spans="1:7">
+    <row r="230" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>235</v>
       </c>
@@ -10838,7 +10855,7 @@
         <v>702</v>
       </c>
     </row>
-    <row r="231" spans="1:7">
+    <row r="231" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>236</v>
       </c>
@@ -10861,7 +10878,7 @@
         <v>703</v>
       </c>
     </row>
-    <row r="232" spans="1:7">
+    <row r="232" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>237</v>
       </c>
@@ -10884,7 +10901,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="233" spans="1:7">
+    <row r="233" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>238</v>
       </c>
@@ -10907,7 +10924,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="234" spans="1:7">
+    <row r="234" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>239</v>
       </c>
@@ -10930,7 +10947,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="235" spans="1:7">
+    <row r="235" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>240</v>
       </c>
@@ -10953,7 +10970,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="236" spans="1:7">
+    <row r="236" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>241</v>
       </c>
@@ -10976,7 +10993,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="237" spans="1:7">
+    <row r="237" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
         <v>242</v>
       </c>
@@ -10999,7 +11016,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="238" spans="1:7">
+    <row r="238" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>243</v>
       </c>
@@ -11022,7 +11039,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="239" spans="1:7">
+    <row r="239" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>244</v>
       </c>
@@ -11042,7 +11059,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="240" spans="1:7">
+    <row r="240" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>245</v>
       </c>
@@ -11062,7 +11079,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="241" spans="1:7">
+    <row r="241" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>246</v>
       </c>
@@ -11085,7 +11102,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="242" spans="1:7">
+    <row r="242" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
         <v>247</v>
       </c>
@@ -11108,7 +11125,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="243" spans="1:7">
+    <row r="243" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
         <v>248</v>
       </c>
@@ -11131,7 +11148,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="244" spans="1:7">
+    <row r="244" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>249</v>
       </c>
@@ -11154,7 +11171,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="245" spans="1:7">
+    <row r="245" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
         <v>250</v>
       </c>
@@ -11174,7 +11191,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="246" spans="1:7">
+    <row r="246" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>251</v>
       </c>
@@ -11194,7 +11211,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="247" spans="1:7">
+    <row r="247" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>252</v>
       </c>
@@ -11214,7 +11231,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="248" spans="1:7">
+    <row r="248" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>253</v>
       </c>
@@ -11234,7 +11251,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="249" spans="1:7">
+    <row r="249" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>254</v>
       </c>
@@ -11254,7 +11271,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="250" spans="1:7">
+    <row r="250" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>255</v>
       </c>
@@ -11274,7 +11291,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="251" spans="1:7">
+    <row r="251" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>256</v>
       </c>
@@ -11294,7 +11311,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="252" spans="1:7">
+    <row r="252" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>257</v>
       </c>
@@ -11314,7 +11331,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="253" spans="1:7">
+    <row r="253" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>258</v>
       </c>
@@ -11334,7 +11351,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="254" spans="1:7">
+    <row r="254" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>259</v>
       </c>
@@ -11354,7 +11371,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="255" spans="1:7">
+    <row r="255" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>260</v>
       </c>
@@ -11374,7 +11391,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="256" spans="1:7">
+    <row r="256" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>261</v>
       </c>

</xml_diff>